<commit_message>
Add Outlook processing audit report
</commit_message>
<xml_diff>
--- a/config/outlook/OAS-K_Outlook-Revisi_Configuration1.xlsx
+++ b/config/outlook/OAS-K_Outlook-Revisi_Configuration1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\outlook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0A449D5-0CB9-455F-AA70-A9E79C5B0D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBEAA6B-EF2D-4E98-A445-17888790808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -722,21 +722,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -765,6 +750,21 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -943,18 +943,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -993,7 +993,7 @@
       <c r="A7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="24" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1015,7 +1015,7 @@
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="23" t="s">
         <v>115</v>
       </c>
       <c r="C9" s="6" t="s">
@@ -1026,7 +1026,7 @@
       <c r="A10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="22" t="s">
         <v>109</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -1037,7 +1037,7 @@
       <c r="A11" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="25" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="6" t="s">
@@ -1048,7 +1048,7 @@
       <c r="A12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="25" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -1135,7 +1135,7 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" sqref="B13:B14" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
@@ -1166,32 +1166,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
     </row>
     <row r="2" spans="1:7" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-    </row>
-    <row r="4" spans="1:7" ht="28">
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="26" t="s">
         <v>117</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1200,10 +1200,10 @@
       <c r="D4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="F4" s="30" t="s">
         <v>119</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -1214,7 +1214,7 @@
       <c r="A5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="31" t="s">
         <v>122</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1223,7 +1223,7 @@
       <c r="D5" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="E5" s="31" t="s">
         <v>122</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -1237,7 +1237,7 @@
       <c r="A6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="32"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -1248,7 +1248,7 @@
       <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="32"/>
+      <c r="B7" s="27"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -1257,7 +1257,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4"/>
-      <c r="B8" s="32"/>
+      <c r="B8" s="27"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4"/>
-      <c r="B9" s="32"/>
+      <c r="B9" s="27"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4"/>
-      <c r="B10" s="32"/>
+      <c r="B10" s="27"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -1284,7 +1284,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="4"/>
-      <c r="B11" s="32"/>
+      <c r="B11" s="27"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -1293,7 +1293,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="4"/>
-      <c r="B12" s="32"/>
+      <c r="B12" s="27"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -1302,7 +1302,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="4"/>
-      <c r="B13" s="32"/>
+      <c r="B13" s="27"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="4"/>
-      <c r="B14" s="32"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -1320,7 +1320,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="4"/>
-      <c r="B15" s="32"/>
+      <c r="B15" s="27"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
@@ -1329,7 +1329,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="4"/>
-      <c r="B16" s="32"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4"/>
-      <c r="B17" s="32"/>
+      <c r="B17" s="27"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4"/>
-      <c r="B18" s="32"/>
+      <c r="B18" s="27"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
@@ -1356,7 +1356,7 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4"/>
-      <c r="B19" s="32"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
@@ -1365,7 +1365,7 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="4"/>
-      <c r="B20" s="32"/>
+      <c r="B20" s="27"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="4"/>
-      <c r="B21" s="32"/>
+      <c r="B21" s="27"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4"/>
-      <c r="B22" s="32"/>
+      <c r="B22" s="27"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
@@ -1392,7 +1392,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="4"/>
-      <c r="B23" s="32"/>
+      <c r="B23" s="27"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
@@ -1401,7 +1401,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4"/>
-      <c r="B24" s="32"/>
+      <c r="B24" s="27"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
@@ -1410,7 +1410,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4"/>
-      <c r="B25" s="32"/>
+      <c r="B25" s="27"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
@@ -1419,7 +1419,7 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="4"/>
-      <c r="B26" s="32"/>
+      <c r="B26" s="27"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -1428,7 +1428,7 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="4"/>
-      <c r="B27" s="32"/>
+      <c r="B27" s="27"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
@@ -1437,7 +1437,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="4"/>
-      <c r="B28" s="32"/>
+      <c r="B28" s="27"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="4"/>
-      <c r="B29" s="32"/>
+      <c r="B29" s="27"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -1455,7 +1455,7 @@
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="4"/>
-      <c r="B30" s="32"/>
+      <c r="B30" s="27"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="4"/>
-      <c r="B31" s="32"/>
+      <c r="B31" s="27"/>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="4"/>
-      <c r="B32" s="32"/>
+      <c r="B32" s="27"/>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="4"/>
-      <c r="B33" s="32"/>
+      <c r="B33" s="27"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="4"/>
-      <c r="B34" s="32"/>
+      <c r="B34" s="27"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="4"/>
-      <c r="B35" s="32"/>
+      <c r="B35" s="27"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
@@ -1509,7 +1509,7 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="4"/>
-      <c r="B36" s="32"/>
+      <c r="B36" s="27"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
@@ -1518,7 +1518,7 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="4"/>
-      <c r="B37" s="32"/>
+      <c r="B37" s="27"/>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
@@ -1527,7 +1527,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="4"/>
-      <c r="B38" s="32"/>
+      <c r="B38" s="27"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
@@ -1536,7 +1536,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="4"/>
-      <c r="B39" s="32"/>
+      <c r="B39" s="27"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="4"/>
-      <c r="B40" s="32"/>
+      <c r="B40" s="27"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
@@ -1554,7 +1554,7 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="4"/>
-      <c r="B41" s="32"/>
+      <c r="B41" s="27"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
@@ -1563,7 +1563,7 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="4"/>
-      <c r="B42" s="32"/>
+      <c r="B42" s="27"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="4"/>
-      <c r="B43" s="32"/>
+      <c r="B43" s="27"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
@@ -1581,7 +1581,7 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="4"/>
-      <c r="B44" s="32"/>
+      <c r="B44" s="27"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="4"/>
-      <c r="B45" s="32"/>
+      <c r="B45" s="27"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="4"/>
-      <c r="B46" s="32"/>
+      <c r="B46" s="27"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
@@ -1608,7 +1608,7 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="4"/>
-      <c r="B47" s="32"/>
+      <c r="B47" s="27"/>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
@@ -1617,7 +1617,7 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="4"/>
-      <c r="B48" s="32"/>
+      <c r="B48" s="27"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="49" spans="1:7">
       <c r="A49" s="4"/>
-      <c r="B49" s="32"/>
+      <c r="B49" s="27"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
@@ -1635,11 +1635,11 @@
     </row>
     <row r="50" spans="1:7">
       <c r="A50" s="7"/>
-      <c r="B50" s="32"/>
+      <c r="B50" s="27"/>
       <c r="C50" s="8"/>
       <c r="D50" s="8"/>
-      <c r="E50" s="32"/>
-      <c r="F50" s="32"/>
+      <c r="E50" s="27"/>
+      <c r="F50" s="27"/>
       <c r="G50" s="9"/>
     </row>
   </sheetData>
@@ -1647,11 +1647,14 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" sqref="A5:B50 E5" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{52E72A51-6698-4921-8CCD-357F3F9B700F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1673,57 +1676,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
     </row>
     <row r="2" spans="1:9" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="E4" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="H4" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="I4" s="33" t="s">
+      <c r="I4" s="28" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1737,7 +1740,7 @@
       <c r="C5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="29" t="s">
         <v>120</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1746,10 +1749,10 @@
       <c r="F5" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="G5" s="34" t="s">
+      <c r="G5" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="34" t="s">
+      <c r="H5" s="29" t="s">
         <v>121</v>
       </c>
       <c r="I5" s="21" t="s">
@@ -4448,11 +4451,11 @@
       <c r="A250" s="7"/>
       <c r="B250" s="8"/>
       <c r="C250" s="8"/>
-      <c r="D250" s="32"/>
+      <c r="D250" s="27"/>
       <c r="E250" s="8"/>
       <c r="F250" s="8"/>
-      <c r="G250" s="32"/>
-      <c r="H250" s="32"/>
+      <c r="G250" s="27"/>
+      <c r="H250" s="27"/>
       <c r="I250" s="9"/>
     </row>
   </sheetData>
@@ -4480,18 +4483,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -4624,18 +4627,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
@@ -4769,20 +4772,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:4" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
@@ -5041,24 +5044,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.649999999999999" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="22.65" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
@@ -5177,14 +5180,14 @@
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="29.4" customHeight="1">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="34" t="s">
         <v>108</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="26"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4"/>

</xml_diff>

<commit_message>
Improve HRIS and Outlook automation workflows
</commit_message>
<xml_diff>
--- a/config/outlook/OAS-K_Outlook-Revisi_Configuration1.xlsx
+++ b/config/outlook/OAS-K_Outlook-Revisi_Configuration1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\outlook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBEAA6B-EF2D-4E98-A445-17888790808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354D0BE9-81AB-43AA-9C62-A3556FA4EABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,52 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="134">
+  <si>
+    <t>Outlook - Revisi | HO Sender Master</t>
+  </si>
+  <si>
+    <t>Master pengirim HO untuk Module Outlook - Revisi. Sender harus cocok dengan Sender_Email dan CC wajib diambil dari Required_CC_Email.</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Nik_Sender</t>
+  </si>
+  <si>
+    <t>Sender_Name</t>
+  </si>
+  <si>
+    <t>Sender_Email</t>
+  </si>
+  <si>
+    <t>Nik_Spv</t>
+  </si>
+  <si>
+    <t>Name_SPV</t>
+  </si>
+  <si>
+    <t>Required_CC_Email</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>20000031815</t>
+  </si>
+  <si>
+    <t>ZULKARNAIN</t>
+  </si>
+  <si>
+    <t>tecnozs013@gmail.com</t>
+  </si>
+  <si>
+    <t>psilang</t>
+  </si>
+  <si>
+    <t>kiyanresto@gmail.com</t>
+  </si>
   <si>
     <t>OAS-K Outlook - Revisi Configuration</t>
   </si>
@@ -55,7 +100,10 @@
     <t>Mailbox_SMTP</t>
   </si>
   <si>
-    <t>Mailbox khusus yang dibaca. Jangan menggunakan default Inbox.</t>
+    <t>karina.hr.1@oto.co.id</t>
+  </si>
+  <si>
+    <t>Shared mailbox yang dibaca melalui Outlook COM.</t>
   </si>
   <si>
     <t>Source_Folder</t>
@@ -70,18 +118,54 @@
     <t>Reply_From_SMTP</t>
   </si>
   <si>
-    <t>Semua balasan dan email summary wajib dikirim dari akun ini.</t>
+    <t>Alamat From untuk balasan dan email summary.</t>
+  </si>
+  <si>
+    <t>Send_Transport</t>
+  </si>
+  <si>
+    <t>SMTP</t>
+  </si>
+  <si>
+    <t>SMTP = relay internal; OUTLOOK = akun Outlook dengan izin Send As.</t>
+  </si>
+  <si>
+    <t>SMTP_Server</t>
+  </si>
+  <si>
+    <t>mail.oto.co.id</t>
+  </si>
+  <si>
+    <t>Server SMTP relay internal yang digunakan VBA/CDO.</t>
+  </si>
+  <si>
+    <t>SMTP_Port</t>
+  </si>
+  <si>
+    <t>Port SMTP relay internal.</t>
+  </si>
+  <si>
+    <t>SMTP_Timeout_Seconds</t>
+  </si>
+  <si>
+    <t>Batas waktu koneksi SMTP dalam detik.</t>
   </si>
   <si>
     <t>Processed_Folder</t>
   </si>
   <si>
+    <t>Deleted</t>
+  </si>
+  <si>
     <t>Email asli dipindahkan ke Deleted Items setelah balasan berhasil dikirim.</t>
   </si>
   <si>
     <t>Output_Root</t>
   </si>
   <si>
+    <t>D:\Python Project\OfficeAutomationSuite-Karina\output</t>
+  </si>
+  <si>
     <t>Folder utama output Outlook - Revisi sebelum dipisahkan menjadi HO dan Branch.</t>
   </si>
   <si>
@@ -151,30 +235,12 @@
     <t>Window_Title</t>
   </si>
   <si>
+    <t>OAS-K | Outlook - Revisi</t>
+  </si>
+  <si>
     <t>Judul jendela module yang terlihat oleh pengguna.</t>
   </si>
   <si>
-    <t>Outlook - Revisi | HO Sender Master</t>
-  </si>
-  <si>
-    <t>Master pengirim HO untuk Module Outlook - Revisi. Sender harus cocok dengan Sender_Email dan CC wajib diambil dari Required_CC_Email.</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Sender_Name</t>
-  </si>
-  <si>
-    <t>Sender_Email</t>
-  </si>
-  <si>
-    <t>Required_CC_Email</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>Outlook - Revisi | Branch Sender Master</t>
   </si>
   <si>
@@ -191,6 +257,15 @@
   </si>
   <si>
     <t>AMU</t>
+  </si>
+  <si>
+    <t>2000031815</t>
+  </si>
+  <si>
+    <t>zulkarnain</t>
+  </si>
+  <si>
+    <t>pislang</t>
   </si>
   <si>
     <t>Outlook - Revisi | Subject Rules</t>
@@ -387,51 +462,6 @@
   </si>
   <si>
     <t>Placeholder utama: {SENDER_NAME}, {PERIOD}, {ORIGINAL_SUBJECT}, {REQUIRED_CC_EMAIL}, {RESUBMIT_DEADLINE}, {ERROR_REASON}, {TOTAL_EMAIL}, {SUCCESS_EMAIL}, {FAILED_EMAIL}, {OUTPUT_TXT_COUNT}, {OUTPUT_FOLDER}</t>
-  </si>
-  <si>
-    <t>D:\Python Project\OfficeAutomationSuite-Karina\output</t>
-  </si>
-  <si>
-    <t>zulkarnainsidik@gmail.com</t>
-  </si>
-  <si>
-    <t>tecnozs013@gmail.com</t>
-  </si>
-  <si>
-    <t>kiyanresto@gmail.com</t>
-  </si>
-  <si>
-    <t>ZULKARNAIN</t>
-  </si>
-  <si>
-    <t>zulkarnain</t>
-  </si>
-  <si>
-    <t>Deleted</t>
-  </si>
-  <si>
-    <t>OAS-K | Outlook - Revisi</t>
-  </si>
-  <si>
-    <t>Nik_Sender</t>
-  </si>
-  <si>
-    <t>Nik_Spv</t>
-  </si>
-  <si>
-    <t>Name_SPV</t>
-  </si>
-  <si>
-    <t>2000031815</t>
-  </si>
-  <si>
-    <t>pislang</t>
-  </si>
-  <si>
-    <t>20000031815</t>
-  </si>
-  <si>
-    <t>psilang</t>
   </si>
 </sst>
 </file>
@@ -654,11 +684,11 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14"/>
   </cellStyleXfs>
   <cellXfs count="37">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -671,7 +701,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -692,10 +722,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -713,59 +743,57 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -934,7 +962,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -944,191 +972,236 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+        <v>15</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>1</v>
+      <c r="A2" s="34" t="s">
+        <v>16</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="10" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="10" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="10" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="10" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>115</v>
+        <v>31</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="28">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>109</v>
+        <v>34</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>35</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>20</v>
+        <v>37</v>
+      </c>
+      <c r="B11" s="20">
+        <v>25</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>23</v>
+        <v>39</v>
+      </c>
+      <c r="B12" s="20">
+        <v>30</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>26</v>
+        <v>41</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>42</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="28">
       <c r="A14" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>29</v>
+        <v>44</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>45</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="28">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="28" customHeight="1">
       <c r="A15" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>110</v>
+        <v>47</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>48</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="12"/>
+        <v>50</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>51</v>
+      </c>
       <c r="C16" s="6" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="13">
+      <c r="A17" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="28">
+      <c r="A19" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="13">
         <v>10000</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>116</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>41</v>
-      </c>
+      <c r="C21" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="B24" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1144,8 +1217,8 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{64215ADF-6FDC-47B6-A0C8-4052ECBB0AC2}"/>
-    <hyperlink ref="B8" r:id="rId2" xr:uid="{7661BB7E-C548-46AF-92B0-8BBBE4AF27F7}"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1167,18 +1240,18 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
+        <v>0</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>43</v>
+      <c r="A2" s="34" t="s">
+        <v>1</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
@@ -1189,53 +1262,53 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>117</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>118</v>
+        <v>6</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>119</v>
+        <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>112</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="5"/>
@@ -1246,7 +1319,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B7" s="27"/>
       <c r="C7" s="5"/>
@@ -1644,8 +1717,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" sqref="A5:B50 E5" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -1653,7 +1726,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" xr:uid="{52E72A51-6698-4921-8CCD-357F3F9B700F}"/>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1677,20 +1750,20 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
+        <v>71</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
     </row>
     <row r="2" spans="1:9" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>50</v>
+      <c r="A2" s="34" t="s">
+        <v>72</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
@@ -1703,65 +1776,65 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="28" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>117</v>
+        <v>3</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="G4" s="28" t="s">
-        <v>118</v>
+        <v>6</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>119</v>
+        <v>7</v>
       </c>
       <c r="I4" s="28" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="28">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="28" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="I5" s="21" t="s">
-        <v>112</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1774,7 +1847,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -4484,49 +4557,49 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+        <v>80</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>56</v>
+      <c r="A2" s="34" t="s">
+        <v>81</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4628,49 +4701,49 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+        <v>88</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
     </row>
     <row r="2" spans="1:3" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>64</v>
+      <c r="A2" s="34" t="s">
+        <v>89</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>66</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4773,15 +4846,15 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+        <v>93</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="2" spans="1:4" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>69</v>
+      <c r="A2" s="34" t="s">
+        <v>94</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
@@ -4789,114 +4862,114 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -5045,17 +5118,17 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.649999999999999" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+        <v>110</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="22.65" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>86</v>
+      <c r="A2" s="34" t="s">
+        <v>111</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
@@ -5065,102 +5138,102 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="100" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="100" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="100" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="100" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -5180,14 +5253,14 @@
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="29.4" customHeight="1">
-      <c r="A11" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
+      <c r="A11" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4"/>
@@ -5263,9 +5336,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" sqref="A5:A20" xr:uid="{00000000-0002-0000-0600-000000000000}">

</xml_diff>